<commit_message>
fix: diccionario con columnas Categoria/Codigo/Definicion con tildes (formato validador IA)
</commit_message>
<xml_diff>
--- a/examples/diccionario_codigos_tesistas.xlsx
+++ b/examples/diccionario_codigos_tesistas.xlsx
@@ -14,13 +14,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
-    <t xml:space="preserve">category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">definition</t>
+    <t xml:space="preserve">Categoría</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definición</t>
   </si>
   <si>
     <t xml:space="preserve">Factores personales</t>

</xml_diff>